<commit_message>
Switch all financials from QAR to Saudi Riyals (SAR)
Every currency figure across the app — fund NAV/IRR/committed/drawn
capital, capital calls and distributions, discount-approval math, model
editor workbooks (built-from-scratch and vibe-coded), reporting/board
letters, ERP figures, ERP integration labels, ASM assumption fields,
ai-generated file content, ec. — now reads in SAR instead of QAR.
Spelled-out currency mentions ("Qatari Riyals") are updated too.

The two demo PDFs and the sample master-model Excel workbook in
demo-assets/ are patched the same way so an uploaded/downloaded sample
document matches the live app's currency.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZjNDFW9f6Aku3qPQR9exQ
</commit_message>
<xml_diff>
--- a/bohio-workspace/demo-assets/Fund_II_Master_Financial_Model.xlsx
+++ b/bohio-workspace/demo-assets/Fund_II_Master_Financial_Model.xlsx
@@ -401,7 +401,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Avg achieved QAR/sqft</t>
+          <t xml:space="preserve">Avg achieved SAR/sqft</t>
         </is>
       </c>
       <c r="B8">
@@ -450,7 +450,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sales proceeds QAR M</t>
+          <t xml:space="preserve">Sales proceeds SAR M</t>
         </is>
       </c>
       <c r="B9">
@@ -499,7 +499,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cumulative proceeds QAR M</t>
+          <t xml:space="preserve">Cumulative proceeds SAR M</t>
         </is>
       </c>
       <c r="B10">
@@ -555,7 +555,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fund consolidated cashflow (QAR M)</t>
+          <t xml:space="preserve">Fund consolidated cashflow (SAR M)</t>
         </is>
       </c>
     </row>
@@ -1060,7 +1060,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Distribution waterfall (QAR M)</t>
+          <t xml:space="preserve">Distribution waterfall (SAR M)</t>
         </is>
       </c>
     </row>
@@ -1122,7 +1122,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">QAR 540M</t>
+          <t xml:space="preserve">SAR 540M</t>
         </is>
       </c>
       <c r="D5">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">QAR 173M</t>
+          <t xml:space="preserve">SAR 173M</t>
         </is>
       </c>
       <c r="D6">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">QAR 43M</t>
+          <t xml:space="preserve">SAR 43M</t>
         </is>
       </c>
       <c r="D7">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">QAR M</t>
+          <t xml:space="preserve">SAR M</t>
         </is>
       </c>
     </row>
@@ -1607,7 +1607,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">QAR M</t>
+          <t xml:space="preserve">SAR M</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1622,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">QAR M</t>
+          <t xml:space="preserve">SAR M</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1757,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">QAR M</t>
+          <t xml:space="preserve">SAR M</t>
         </is>
       </c>
     </row>
@@ -1831,7 +1831,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Portfolio rollup by asset (QAR M)</t>
+          <t xml:space="preserve">Portfolio rollup by asset (SAR M)</t>
         </is>
       </c>
     </row>
@@ -2093,7 +2093,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">QAR M</t>
+          <t xml:space="preserve">SAR M</t>
         </is>
       </c>
     </row>
@@ -2352,7 +2352,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marina Tower — asset cashflow (QAR M)</t>
+          <t xml:space="preserve">Marina Tower — asset cashflow (SAR M)</t>
         </is>
       </c>
     </row>
@@ -3207,7 +3207,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ash Shati Residences — asset cashflow (QAR M)</t>
+          <t xml:space="preserve">Ash Shati Residences — asset cashflow (SAR M)</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rawdah Plaza — asset cashflow (QAR M)</t>
+          <t xml:space="preserve">Rawdah Plaza — asset cashflow (SAR M)</t>
         </is>
       </c>
     </row>
@@ -4917,7 +4917,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rayyan Block — asset cashflow (QAR M)</t>
+          <t xml:space="preserve">Rayyan Block — asset cashflow (SAR M)</t>
         </is>
       </c>
     </row>
@@ -5772,7 +5772,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nahdah Logistics — asset cashflow (QAR M)</t>
+          <t xml:space="preserve">Nahdah Logistics — asset cashflow (SAR M)</t>
         </is>
       </c>
     </row>
@@ -6627,7 +6627,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Andalus Quarter — asset cashflow (QAR M)</t>
+          <t xml:space="preserve">Andalus Quarter — asset cashflow (SAR M)</t>
         </is>
       </c>
     </row>
@@ -7482,7 +7482,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fund debt schedule (QAR M)</t>
+          <t xml:space="preserve">Fund debt schedule (SAR M)</t>
         </is>
       </c>
     </row>

</xml_diff>